<commit_message>
Removed GRPC and multi-region
</commit_message>
<xml_diff>
--- a/public/simwood/port-in-template.xlsx
+++ b/public/simwood/port-in-template.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Port-In Template" sheetId="1" r:id="rId1"/>
+    <sheet name="Port In" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R3"/>
+  <dimension ref="A1:R1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -449,127 +449,15 @@
         <v>Contact Email</v>
       </c>
       <c r="Q1" t="str">
-        <v>Line Type</v>
+        <v>Is Multi Line</v>
       </c>
       <c r="R1" t="str">
         <v>PAC</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>442033001234</v>
-      </c>
-      <c r="B2" t="str">
-        <v>local</v>
-      </c>
-      <c r="C2" t="str">
-        <v>442033009999</v>
-      </c>
-      <c r="D2" t="str">
-        <v>ACCT-1001</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Example Telecom</v>
-      </c>
-      <c r="F2" t="str">
-        <v>001</v>
-      </c>
-      <c r="G2" t="str">
-        <v>10</v>
-      </c>
-      <c r="H2" t="str">
-        <v>5</v>
-      </c>
-      <c r="I2" t="str">
-        <v>Akhil</v>
-      </c>
-      <c r="J2" t="str">
-        <v>Kumar</v>
-      </c>
-      <c r="K2" t="str">
-        <v>12A</v>
-      </c>
-      <c r="L2" t="str">
-        <v>High Street</v>
-      </c>
-      <c r="M2" t="str">
-        <v>London</v>
-      </c>
-      <c r="N2" t="str">
-        <v>SW1A 1AA</v>
-      </c>
-      <c r="O2" t="str">
-        <v>442033001235,442033001236</v>
-      </c>
-      <c r="P2" t="str">
-        <v>ops@example.com</v>
-      </c>
-      <c r="Q2" t="str">
-        <v>multiline</v>
-      </c>
-      <c r="R2" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>447700900123</v>
-      </c>
-      <c r="B3" t="str">
-        <v>mobile</v>
-      </c>
-      <c r="C3" t="str">
-        <v/>
-      </c>
-      <c r="D3" t="str">
-        <v/>
-      </c>
-      <c r="E3" t="str">
-        <v/>
-      </c>
-      <c r="F3" t="str">
-        <v/>
-      </c>
-      <c r="G3" t="str">
-        <v/>
-      </c>
-      <c r="H3" t="str">
-        <v/>
-      </c>
-      <c r="I3" t="str">
-        <v/>
-      </c>
-      <c r="J3" t="str">
-        <v/>
-      </c>
-      <c r="K3" t="str">
-        <v/>
-      </c>
-      <c r="L3" t="str">
-        <v/>
-      </c>
-      <c r="M3" t="str">
-        <v/>
-      </c>
-      <c r="N3" t="str">
-        <v/>
-      </c>
-      <c r="O3" t="str">
-        <v/>
-      </c>
-      <c r="P3" t="str">
-        <v/>
-      </c>
-      <c r="Q3" t="str">
-        <v/>
-      </c>
-      <c r="R3" t="str">
-        <v>ABC123456</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:R3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:R1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>